<commit_message>
edim-ai-blueprint: DB 스키마·API 교차 검증 → DB v0.2 (50테이블) + API 80
검증: FK 무결성 NONE, 기능↔스키마 참조 NONE, 보완노트 후보 4종 미반영 발견 → 반영
- DB v0.2: dwg_supersedure·doc_control·prt_supplier_code_map·erp_warehouse 추가,
  mat_material.hazard_class·tbx_ui_form.head_key 컬럼, 공통코드 2그룹 (46→50테이블/435컬럼)
- API 68→80: referencers/variants/supersede, doc-controls(문서함·status·채번),
  codes excel import/export, BOM export, supplier-code-maps, QR issue/resolve
- 기능정의서 DB 참조 신규 테이블로 갱신 (DOC/DWG-027/ERP-018/020), RTM 재생성 178/178
- 보완노트 §3.1 반영 완료 표시, 산출물목록·README·개요 버전 갱신
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_기능정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_기능정의서.xlsx
@@ -1991,7 +1991,7 @@
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>dwg_file, sys_approval_request</t>
+          <t>doc_control</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>sys_role_permission</t>
+          <t>doc_control, sys_role_permission</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>doc_control</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="J68" s="8" t="inlineStr">
         <is>
-          <t>dwg_revision</t>
+          <t>dwg_supersedure, dwg_revision</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
@@ -8575,7 +8575,7 @@
       </c>
       <c r="J139" s="8" t="inlineStr">
         <is>
-          <t>prt_part, com_company</t>
+          <t>prt_supplier_code_map</t>
         </is>
       </c>
       <c r="K139" s="6" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="J141" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>erp_warehouse, mat_material</t>
         </is>
       </c>
       <c r="K141" s="6" t="inlineStr">
@@ -8705,7 +8705,7 @@
       </c>
       <c r="L141" s="8" t="inlineStr">
         <is>
-          <t>슬라이드 46 — 상세 테이블 v0.2</t>
+          <t>슬라이드 46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
edim-ai-blueprint: DB·API 설계 품질 리뷰 — DB v0.3 (6결함 수정, 53테이블) + API 95
DB 설계 결함 수정:
1) erp_process_def.prev/next_codes CSV → erp_process_edge 테이블 + 대리키 표준화
2) tbl_data_row.row_key_num 추가 — VARCHAR 사전순으로 Macro 숫자 범위(10:25) 조회 불가 결함
3) 한글 enum CHECK 13곳 → 영문 코드 (i18n REQ-N-015, 코드 값 원칙 명문화)
4) sys_tenant 마스터 신설 (tenant_id 참조 대상 부재)
5) code_relationship.match_condition JSONB → slot_map 정규 테이블 (BOM 전개 조인·검증 가능)
6) sys_user.login_id 테넌트 범위 UQ
+ XOR 제약 3건(dim binding·price target·supplier map), cst_price 기간 배타(EXCLUDE gist),
  Hierarchy 이동·JSONB 경계 지침, slot_values JSONB 유지 결정 기록

API 80→95: users/roles/tenants, hierarchy 수정/삭제, parts/materials, dimensions PATCH,
selections 목록, projects 등록/목록, process-defs 생성/수정
연쇄: 기능·요구사항·화면설계서 match_condition 표기 정리, RTM 178/178 유지, 회귀 검증 클린
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_기능정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_기능정의서.xlsx
@@ -2604,7 +2604,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>match_condition으로 Mother/Child 자릿수 연동</t>
+          <t>Slot 매핑 테이블(slot_map)로 Mother/Child 자릿수 연동</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>code_relationship</t>
+          <t>code_relationship, code_relationship_slot_map</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -10635,7 +10635,7 @@
       </c>
       <c r="J175" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>sys_tenant</t>
         </is>
       </c>
       <c r="K175" s="6" t="inlineStr">

</xml_diff>